<commit_message>
feat: integrate 6 factions (Gen Red, Trauma Team, Piranhas, Wild Things, Tyger Claws, Maelstrom) + extraction docs
Supabase changes:
- Gen Red: 6 profile corrections (Apex, Hi-Stick, Tetra)
- Trauma Team: 5 corrections + Doc Salvage Elite + 3 new lineages (EMT Lead, EMR Pilot, Security Gunner)
- Piranhas: 5 new lineages (Block Boss, Chuckles, Headbanger, Mr/Ms Reveler) + multi-faction Piranha/Zoner/Bozo
- Wild Things: 6 new lineages (Whirly Girl, Baby Face, Bruiser, Brutalizer, Showfur, Bouncer)
- Tyger Claws: extraction docs
- Maelstrom: Berserker cost 8→18, Hammerlord Vet tokens fix, Flenser Base cost 15→20, Warlord SMG range fix, Ranged Specialist type→Specialist, new Intimidator + Iron Throw weapon

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Updated Gears and Weapons.xlsx
+++ b/Updated Gears and Weapons.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielherbera/Dropbox/Antigravity/Cyberpunk Combat Zone/combat-zone-companion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7125CBCF-DB2D-C04F-82B1-3E853AFDFD7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D1BBB06-5FE2-A44F-84FC-8B414F6C6550}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="800" yWindow="1020" windowWidth="25040" windowHeight="15020" xr2:uid="{2D559F39-C472-A142-940A-323FAC874AD6}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1912" uniqueCount="662">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1915" uniqueCount="661">
   <si>
     <t>Name</t>
   </si>
@@ -1821,9 +1821,6 @@
   </si>
   <si>
     <t>Steroid Pack</t>
-  </si>
-  <si>
-    <t>M</t>
   </si>
   <si>
     <t>Target friendly model may make a YELLOW move for free and then make a Basic Melee Attack with +1 to the roll for free.</t>
@@ -3371,6 +3368,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{07BA0805-9A57-C24E-887F-3D529B9F61D3}">
+  <we:reference id="wa200009404" version="1.0.0.5" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="wa200009404" version="1.0.0.5" store="en-US" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="Office.AutoShowTaskpaneWithDocument" value="true"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6BAC5D4-0582-D247-8705-5BCAFDFF9DD1}">
   <dimension ref="A1:AY264"/>
@@ -3857,9 +3876,7 @@
       <c r="G6" s="95"/>
       <c r="H6" s="96"/>
       <c r="I6" s="93"/>
-      <c r="J6" s="94" t="s">
-        <v>37</v>
-      </c>
+      <c r="J6" s="94"/>
       <c r="K6" s="95"/>
       <c r="L6" s="96"/>
       <c r="M6" s="97"/>
@@ -20308,7 +20325,9 @@
       <c r="F222" s="95"/>
       <c r="G222" s="95"/>
       <c r="H222" s="96"/>
-      <c r="I222" s="93"/>
+      <c r="I222" s="93" t="s">
+        <v>37</v>
+      </c>
       <c r="J222" s="94"/>
       <c r="K222" s="95"/>
       <c r="L222" s="96"/>
@@ -21140,8 +21159,8 @@
       <c r="D232" s="91" t="s">
         <v>31</v>
       </c>
-      <c r="E232" s="91" t="s">
-        <v>589</v>
+      <c r="E232" s="95" t="s">
+        <v>58</v>
       </c>
       <c r="F232" s="91"/>
       <c r="G232" s="91"/>
@@ -21157,7 +21176,7 @@
       <c r="O232" s="96"/>
       <c r="P232" s="98"/>
       <c r="Q232" s="99" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="R232" s="100" t="s">
         <v>121</v>
@@ -21210,7 +21229,7 @@
     </row>
     <row r="233" spans="1:51" ht="27" x14ac:dyDescent="0.2">
       <c r="A233" s="103" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B233" s="104" t="s">
         <v>30</v>
@@ -21232,7 +21251,7 @@
       <c r="O233" s="96"/>
       <c r="P233" s="98"/>
       <c r="Q233" s="105" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="R233" s="106" t="s">
         <v>121</v>
@@ -21303,7 +21322,7 @@
     </row>
     <row r="234" spans="1:51" x14ac:dyDescent="0.2">
       <c r="A234" s="89" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="B234" s="90" t="s">
         <v>30</v>
@@ -21327,7 +21346,7 @@
       <c r="O234" s="96"/>
       <c r="P234" s="98"/>
       <c r="Q234" s="99" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="R234" s="100"/>
       <c r="S234" s="101">
@@ -21372,7 +21391,7 @@
     </row>
     <row r="235" spans="1:51" ht="27" x14ac:dyDescent="0.2">
       <c r="A235" s="103" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B235" s="104" t="s">
         <v>69</v>
@@ -21398,7 +21417,7 @@
       <c r="O235" s="96"/>
       <c r="P235" s="98"/>
       <c r="Q235" s="105" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="R235" s="106"/>
       <c r="S235" s="94" t="s">
@@ -21443,7 +21462,7 @@
     </row>
     <row r="236" spans="1:51" x14ac:dyDescent="0.2">
       <c r="A236" s="89" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B236" s="90" t="s">
         <v>69</v>
@@ -21471,7 +21490,7 @@
       <c r="O236" s="96"/>
       <c r="P236" s="98"/>
       <c r="Q236" s="99" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="R236" s="100"/>
       <c r="S236" s="101" t="s">
@@ -21516,7 +21535,7 @@
     </row>
     <row r="237" spans="1:51" ht="40" x14ac:dyDescent="0.2">
       <c r="A237" s="103" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B237" s="104" t="s">
         <v>30</v>
@@ -21538,7 +21557,7 @@
       <c r="O237" s="96"/>
       <c r="P237" s="98"/>
       <c r="Q237" s="105" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="R237" s="106" t="s">
         <v>46</v>
@@ -21585,7 +21604,7 @@
     </row>
     <row r="238" spans="1:51" ht="40" x14ac:dyDescent="0.2">
       <c r="A238" s="89" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B238" s="90" t="s">
         <v>30</v>
@@ -21607,7 +21626,7 @@
       <c r="O238" s="96"/>
       <c r="P238" s="98"/>
       <c r="Q238" s="99" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="R238" s="100" t="s">
         <v>121</v>
@@ -21654,7 +21673,7 @@
     </row>
     <row r="239" spans="1:51" ht="27" x14ac:dyDescent="0.2">
       <c r="A239" s="103" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B239" s="104" t="s">
         <v>30</v>
@@ -21676,7 +21695,7 @@
       <c r="O239" s="96"/>
       <c r="P239" s="98"/>
       <c r="Q239" s="105" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="R239" s="106" t="s">
         <v>46</v>
@@ -21729,7 +21748,7 @@
     </row>
     <row r="240" spans="1:51" x14ac:dyDescent="0.2">
       <c r="A240" s="89" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B240" s="90" t="s">
         <v>69</v>
@@ -21759,7 +21778,7 @@
       <c r="O240" s="96"/>
       <c r="P240" s="98"/>
       <c r="Q240" s="99" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="R240" s="100"/>
       <c r="S240" s="101" t="s">
@@ -21804,7 +21823,7 @@
     </row>
     <row r="241" spans="1:51" x14ac:dyDescent="0.2">
       <c r="A241" s="103" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B241" s="104" t="s">
         <v>69</v>
@@ -21826,7 +21845,7 @@
       <c r="O241" s="96"/>
       <c r="P241" s="98"/>
       <c r="Q241" s="105" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="R241" s="106"/>
       <c r="S241" s="94" t="s">
@@ -21871,7 +21890,7 @@
     </row>
     <row r="242" spans="1:51" x14ac:dyDescent="0.2">
       <c r="A242" s="89" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B242" s="90" t="s">
         <v>30</v>
@@ -21893,7 +21912,7 @@
       <c r="O242" s="96"/>
       <c r="P242" s="98"/>
       <c r="Q242" s="99" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="R242" s="100" t="s">
         <v>319</v>
@@ -21946,7 +21965,7 @@
     </row>
     <row r="243" spans="1:51" x14ac:dyDescent="0.2">
       <c r="A243" s="103" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B243" s="104" t="s">
         <v>69</v>
@@ -21976,7 +21995,7 @@
       <c r="O243" s="96"/>
       <c r="P243" s="98"/>
       <c r="Q243" s="105" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="R243" s="106"/>
       <c r="S243" s="94" t="s">
@@ -22021,7 +22040,7 @@
     </row>
     <row r="244" spans="1:51" x14ac:dyDescent="0.2">
       <c r="A244" s="89" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="B244" s="90" t="s">
         <v>30</v>
@@ -22051,10 +22070,10 @@
       <c r="O244" s="96"/>
       <c r="P244" s="98"/>
       <c r="Q244" s="99" t="s">
+        <v>613</v>
+      </c>
+      <c r="R244" s="100" t="s">
         <v>614</v>
-      </c>
-      <c r="R244" s="100" t="s">
-        <v>615</v>
       </c>
       <c r="S244" s="101"/>
       <c r="T244" s="101"/>
@@ -22116,7 +22135,7 @@
     </row>
     <row r="245" spans="1:51" ht="40" x14ac:dyDescent="0.2">
       <c r="A245" s="103" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B245" s="104" t="s">
         <v>30</v>
@@ -22140,7 +22159,7 @@
       <c r="O245" s="96"/>
       <c r="P245" s="98"/>
       <c r="Q245" s="105" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="R245" s="106" t="s">
         <v>33</v>
@@ -22187,7 +22206,7 @@
     </row>
     <row r="246" spans="1:51" ht="53" x14ac:dyDescent="0.2">
       <c r="A246" s="89" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="B246" s="90" t="s">
         <v>30</v>
@@ -22213,7 +22232,7 @@
       <c r="O246" s="96"/>
       <c r="P246" s="98"/>
       <c r="Q246" s="99" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="R246" s="100" t="s">
         <v>580</v>
@@ -22260,7 +22279,7 @@
     </row>
     <row r="247" spans="1:51" ht="53" x14ac:dyDescent="0.2">
       <c r="A247" s="103" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B247" s="104" t="s">
         <v>30</v>
@@ -22282,7 +22301,7 @@
       <c r="O247" s="96"/>
       <c r="P247" s="98"/>
       <c r="Q247" s="105" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="R247" s="106"/>
       <c r="S247" s="94"/>
@@ -22327,7 +22346,7 @@
     </row>
     <row r="248" spans="1:51" ht="79" x14ac:dyDescent="0.2">
       <c r="A248" s="89" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B248" s="90" t="s">
         <v>30</v>
@@ -22349,7 +22368,7 @@
       <c r="O248" s="96"/>
       <c r="P248" s="98"/>
       <c r="Q248" s="99" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="R248" s="100"/>
       <c r="S248" s="101"/>
@@ -22394,7 +22413,7 @@
     </row>
     <row r="249" spans="1:51" ht="40" x14ac:dyDescent="0.2">
       <c r="A249" s="103" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="B249" s="104" t="s">
         <v>30</v>
@@ -22416,7 +22435,7 @@
       <c r="O249" s="96"/>
       <c r="P249" s="98"/>
       <c r="Q249" s="105" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="R249" s="106"/>
       <c r="S249" s="94" t="s">
@@ -22461,7 +22480,7 @@
     </row>
     <row r="250" spans="1:51" ht="27" x14ac:dyDescent="0.2">
       <c r="A250" s="89" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B250" s="90" t="s">
         <v>30</v>
@@ -22487,7 +22506,7 @@
       <c r="O250" s="96"/>
       <c r="P250" s="98"/>
       <c r="Q250" s="99" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="R250" s="100" t="s">
         <v>546</v>
@@ -22534,7 +22553,7 @@
     </row>
     <row r="251" spans="1:51" x14ac:dyDescent="0.2">
       <c r="A251" s="103" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B251" s="104" t="s">
         <v>69</v>
@@ -22560,7 +22579,7 @@
       <c r="O251" s="96"/>
       <c r="P251" s="98"/>
       <c r="Q251" s="105" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="R251" s="106"/>
       <c r="S251" s="94" t="s">
@@ -22605,7 +22624,7 @@
     </row>
     <row r="252" spans="1:51" ht="27" x14ac:dyDescent="0.2">
       <c r="A252" s="89" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B252" s="90" t="s">
         <v>30</v>
@@ -22627,7 +22646,7 @@
       <c r="O252" s="96"/>
       <c r="P252" s="98"/>
       <c r="Q252" s="99" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R252" s="100" t="s">
         <v>213</v>
@@ -22674,7 +22693,7 @@
     </row>
     <row r="253" spans="1:51" ht="27" x14ac:dyDescent="0.2">
       <c r="A253" s="103" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B253" s="104" t="s">
         <v>30</v>
@@ -22696,7 +22715,7 @@
       <c r="O253" s="96"/>
       <c r="P253" s="98"/>
       <c r="Q253" s="105" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="R253" s="106"/>
       <c r="S253" s="94" t="s">
@@ -22747,7 +22766,7 @@
     </row>
     <row r="254" spans="1:51" x14ac:dyDescent="0.2">
       <c r="A254" s="89" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B254" s="90" t="s">
         <v>30</v>
@@ -22777,10 +22796,10 @@
       <c r="O254" s="96"/>
       <c r="P254" s="98"/>
       <c r="Q254" s="99" t="s">
+        <v>634</v>
+      </c>
+      <c r="R254" s="100" t="s">
         <v>635</v>
-      </c>
-      <c r="R254" s="100" t="s">
-        <v>636</v>
       </c>
       <c r="S254" s="101">
         <v>5</v>
@@ -22836,7 +22855,7 @@
     </row>
     <row r="255" spans="1:51" ht="27" x14ac:dyDescent="0.2">
       <c r="A255" s="103" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B255" s="104" t="s">
         <v>30</v>
@@ -22858,7 +22877,7 @@
       <c r="O255" s="96"/>
       <c r="P255" s="98"/>
       <c r="Q255" s="105" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="R255" s="106" t="s">
         <v>46</v>
@@ -22905,7 +22924,7 @@
     </row>
     <row r="256" spans="1:51" x14ac:dyDescent="0.2">
       <c r="A256" s="89" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="B256" s="90" t="s">
         <v>30</v>
@@ -22935,10 +22954,10 @@
       <c r="O256" s="96"/>
       <c r="P256" s="98"/>
       <c r="Q256" s="99" t="s">
+        <v>639</v>
+      </c>
+      <c r="R256" s="100" t="s">
         <v>640</v>
-      </c>
-      <c r="R256" s="100" t="s">
-        <v>641</v>
       </c>
       <c r="S256" s="101"/>
       <c r="T256" s="101"/>
@@ -22982,7 +23001,7 @@
     </row>
     <row r="257" spans="1:51" ht="66" x14ac:dyDescent="0.2">
       <c r="A257" s="103" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B257" s="104" t="s">
         <v>30</v>
@@ -23004,10 +23023,10 @@
       <c r="O257" s="96"/>
       <c r="P257" s="98"/>
       <c r="Q257" s="105" t="s">
+        <v>642</v>
+      </c>
+      <c r="R257" s="106" t="s">
         <v>643</v>
-      </c>
-      <c r="R257" s="106" t="s">
-        <v>644</v>
       </c>
       <c r="S257" s="94"/>
       <c r="T257" s="94"/>
@@ -23051,7 +23070,7 @@
     </row>
     <row r="258" spans="1:51" ht="40" x14ac:dyDescent="0.2">
       <c r="A258" s="89" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B258" s="90" t="s">
         <v>30</v>
@@ -23073,7 +23092,7 @@
       <c r="O258" s="96"/>
       <c r="P258" s="98"/>
       <c r="Q258" s="99" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="R258" s="100" t="s">
         <v>319</v>
@@ -23120,7 +23139,7 @@
     </row>
     <row r="259" spans="1:51" x14ac:dyDescent="0.2">
       <c r="A259" s="103" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B259" s="104" t="s">
         <v>30</v>
@@ -23142,10 +23161,10 @@
       <c r="O259" s="96"/>
       <c r="P259" s="98"/>
       <c r="Q259" s="105" t="s">
+        <v>647</v>
+      </c>
+      <c r="R259" s="106" t="s">
         <v>648</v>
-      </c>
-      <c r="R259" s="106" t="s">
-        <v>649</v>
       </c>
       <c r="S259" s="94">
         <v>3</v>
@@ -23189,7 +23208,7 @@
     </row>
     <row r="260" spans="1:51" x14ac:dyDescent="0.2">
       <c r="A260" s="89" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B260" s="90" t="s">
         <v>30</v>
@@ -23213,10 +23232,10 @@
       <c r="O260" s="96"/>
       <c r="P260" s="98"/>
       <c r="Q260" s="99" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="R260" s="100" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="S260" s="101" t="s">
         <v>34</v>
@@ -23266,7 +23285,7 @@
     </row>
     <row r="261" spans="1:51" ht="40" x14ac:dyDescent="0.2">
       <c r="A261" s="103" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="B261" s="104" t="s">
         <v>30</v>
@@ -23288,10 +23307,10 @@
       <c r="O261" s="96"/>
       <c r="P261" s="98"/>
       <c r="Q261" s="105" t="s">
+        <v>652</v>
+      </c>
+      <c r="R261" s="106" t="s">
         <v>653</v>
-      </c>
-      <c r="R261" s="106" t="s">
-        <v>654</v>
       </c>
       <c r="S261" s="94"/>
       <c r="T261" s="94"/>
@@ -23335,7 +23354,7 @@
     </row>
     <row r="262" spans="1:51" x14ac:dyDescent="0.2">
       <c r="A262" s="107" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B262" s="108" t="s">
         <v>30</v>
@@ -23350,19 +23369,25 @@
       <c r="F262" s="109"/>
       <c r="G262" s="109"/>
       <c r="H262" s="110"/>
-      <c r="I262" s="93"/>
-      <c r="J262" s="111"/>
-      <c r="K262" s="109"/>
+      <c r="I262" s="93" t="s">
+        <v>37</v>
+      </c>
+      <c r="J262" s="111" t="s">
+        <v>37</v>
+      </c>
+      <c r="K262" s="109" t="s">
+        <v>37</v>
+      </c>
       <c r="L262" s="110"/>
       <c r="M262" s="112"/>
       <c r="N262" s="109"/>
       <c r="O262" s="110"/>
       <c r="P262" s="98"/>
       <c r="Q262" s="113" t="s">
+        <v>655</v>
+      </c>
+      <c r="R262" s="114" t="s">
         <v>656</v>
-      </c>
-      <c r="R262" s="114" t="s">
-        <v>657</v>
       </c>
       <c r="S262" s="111">
         <v>6</v>
@@ -23406,7 +23431,7 @@
     </row>
     <row r="263" spans="1:51" x14ac:dyDescent="0.2">
       <c r="A263" s="115" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="B263" s="116" t="s">
         <v>30</v>
@@ -23436,10 +23461,10 @@
       <c r="O263" s="110"/>
       <c r="P263" s="98"/>
       <c r="Q263" s="119" t="s">
+        <v>658</v>
+      </c>
+      <c r="R263" s="120" t="s">
         <v>659</v>
-      </c>
-      <c r="R263" s="120" t="s">
-        <v>660</v>
       </c>
       <c r="S263" s="121"/>
       <c r="T263" s="121"/>
@@ -23483,7 +23508,7 @@
     </row>
     <row r="264" spans="1:51" ht="27" x14ac:dyDescent="0.2">
       <c r="A264" s="107" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B264" s="108" t="s">
         <v>69</v>

</xml_diff>